<commit_message>
Fixed path in 1a_wrangle_obs_data.R leading to addition of 1 datapoint and reran downstream analysis that was affected by this (no major changes in results)
</commit_message>
<xml_diff>
--- a/Data/processed/n_observed_males.xlsx
+++ b/Data/processed/n_observed_males.xlsx
@@ -693,7 +693,7 @@
         <v>2018</v>
       </c>
       <c r="B25" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C25" t="n">
         <v>1.67</v>
@@ -735,7 +735,7 @@
         <v>2021</v>
       </c>
       <c r="B28" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C28" t="n">
         <v>1.03</v>

</xml_diff>

<commit_message>
fix: correct male count for 2002, rerun pipeline (no significant effect on results)
</commit_message>
<xml_diff>
--- a/Data/processed/n_observed_males.xlsx
+++ b/Data/processed/n_observed_males.xlsx
@@ -469,7 +469,7 @@
         <v>2002</v>
       </c>
       <c r="B9" t="n">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="C9" t="n">
         <v>1.57</v>
@@ -623,7 +623,7 @@
         <v>2013</v>
       </c>
       <c r="B20" t="n">
-        <v>168</v>
+        <v>96</v>
       </c>
       <c r="C20" t="n">
         <v>2.11</v>
@@ -637,7 +637,7 @@
         <v>2014</v>
       </c>
       <c r="B21" t="n">
-        <v>39</v>
+        <v>111</v>
       </c>
       <c r="C21" t="n">
         <v>0.3</v>

</xml_diff>